<commit_message>
Added the project deletion feature and made the company title card in the industry viewed section
</commit_message>
<xml_diff>
--- a/company_leads.xlsx
+++ b/company_leads.xlsx
@@ -8,6 +8,7 @@
   </bookViews>
   <sheets>
     <sheet name="Sheet" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="CodePilot AI" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -566,7 +567,6 @@
           <t>https://www.linkedin.com/company/persistent-systems</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -654,121 +654,1102 @@
           <t>ocean software technologies,I-Bank 4.0,Best Core Banking System,Credit Cooperative Society software,online Credit Cooperative Society CBS software,Multi-State Society Software,Nidhi Company software,banking Software,cooperative society software free download,Credit Cooperative Society software in nagpur,it company nagpur,cbs,web,bfsi companies,VPS,Dedicated,Server,free Credit Society Accounting Loans and Deposits Software,core banking system for microfinance</t>
         </is>
       </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Yogesh Kedar|https://in.linkedin.com/in/yogesh-kedar-65210734</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>https://in.linkedin.com/company/ocean-software-technologies</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>https://in.linkedin.com/in/yogesh-kedar-65210734</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Santosh Selokar Information Technology Pvt.Ltd Nagpur (SSIT.Pvt.Ltd)</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>https://www.ssinfotech.org/</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>+91 96579 59184</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>FCI Housing Society, Plot no 9, Narendra Nagar Extension, New Narendra Nagar, Manish Nagar, Somalwada, Nagpur, Maharashtra 440015, India</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>4.6</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>SSIT</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>santosh selokar|https://in.linkedin.com/in/santosh-selokar-4a62b831</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>https://in.linkedin.com/in/santosh-selokar-b7655618</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>GrowNixt Technologies Pvt. Ltd.</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>IT Park Nagpur IT Park road Gayatri appartment 202, Nagpur, Maharashtra 440022, India</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>4.9</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>rewan gadkari|https://in.linkedin.com/in/rewan-gadkari-883804225</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>https://in.linkedin.com/company/grownixt-technologies</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>https://in.linkedin.com/in/rewan-gadkari-883804225</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>S R solutions</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>https://digitronsoftwares.com/</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>+91 77092 66577</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>2nd FLOOR, 10A, c/o, Main Rd, above SAI ENTERPRIESE, beside CANARA ATM, New Diamond Nagar, Shaktimata Nagar, Nandanvan, Nagpur, Maharashtra 440024, India</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>4.7</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>this is multilingual example meta tag for english</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>digitronsoftwares@gmail.com</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Tessy Anifowoshe sr|https://www.linkedin.com/in/tessy-anifowoshe-sr-9a135a184</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>https://in.linkedin.com/company/sr-solutions-realesateservices</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Pixel Values Technolabs | Software Company</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>https://www.pixelvalues.com/</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>+91 84848 36319</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Swapna Apartment, 35, beside Mantri Sadan, Shivaji Nagar, Nagpur, Maharashtra 440010, India</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>4.8</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Pixel Values is a Best Mobile App Development Company and among the Top Web Development Companies offering custom Android, iOS, and scalable web solutions.</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>info@pixelvalues.com</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Tauseef Anwar|https://in.linkedin.com/in/tauseefanwar</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/pixel-values-techno-labs</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>https://in.linkedin.com/in/tauseefanwar</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Xceller IT Services</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>http://www.xceller.com/</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>+91 93267 44884</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>13/1, Diglin Industries, IT Park Rd, Parsodi, Nagpur, Maharashtra 440022, India</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>4.5</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Discover tailored IT services &amp; solutions at Xceller. From consulting to development, we empower your business with reliable tech expertise and innovation.</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Anshu S|https://in.linkedin.com/in/anshu-s-74bb41217</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>https://au.linkedin.com/company/xcellerate-it</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>https://in.linkedin.com/in/mohit-lanjewar-9199a5294</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Callisto IT Solutions - Best Software Development , Web Application Development and Training &amp; IT InternshipCompany</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>http://www.callistoitsolutions.com/</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>+91 70572 05423</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>4 - Shivshakti App, Bhagwan Nagar Rd, Banarjee Layout, Rameshwari, Nagpur, Maharashtra 440027, India</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>4.4</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Not Available</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>https://in.linkedin.com/company/callisto-it-solutions</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Nass Technologies - Software Development &amp; IT Training</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>http://www.nasstechnologies.com/</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>+91 82372 66913</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>1st Floor, 13, Plot No 5, Borgaon Rd, beside HDFC Bank, near Jafar Nagar, Sugat Colony, Jafar Nagar, Police Line Takli, Nagpur, Maharashtra 440013, India</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>4.6</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Nass Technologies has the most advanced digital solutions for your organisation. Web development and mobile apps are the first steps in digital transformation.</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>info@nasstechnologies.com</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Valivullah Michael|https://www.linkedin.com/in/valivullah-michael-1b337471</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>https://in.linkedin.com/company/nass-technologies</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>TALLYTACT LLP</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>https://www.tallytact.com/</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>+91 93266 47411</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Plot no.80, opp. Nirman Enclave, Gajanan Nagar, Nagpur, Maharashtra 440015, India</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>4.8</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>TALLYTACT LLP is helping Accountant &amp; CAs solving all TallyPrime Release 7.0 related all problems.</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>sales@tallytact.com</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Not Available</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>https://in.linkedin.com/company/tallytact-llp</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>https://in.linkedin.com/in/mayur-tajnekar</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Pegasus Technologies &amp; Software Private Limited Best Data Science analytics institute In Nagpur</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>http://pegasusacademy.in/</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>+91 98235 20987</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Plot No. 43, Mire Layout, Kabir Nagar, Nandanvan, Nagpur, Maharashtra 440009, India</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>4.5</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Pegasus Academy – Training | Certification | Placement</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>Not Available</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>https://in.linkedin.com/company/pegasus-technologies-software-pvt-ltd</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>https://in.linkedin.com/in/komal-tembhare-21b700236</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Radical Global</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>http://www.radicalglobal.net/</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>+91 90212 51392</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>1, Besides Deendayal Uppadhaya Garden, 94, Jawahar Nagar, Raghuji Nagar, Nagpur, Maharashtra 440024, India</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>4.8</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Radical Global – Digital Workplace Services</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Vibhor Khatwar|https://in.linkedin.com/in/vibhor-khatwar-6870485b</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>https://in.linkedin.com/company/radicalglobalcompany</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>https://in.linkedin.com/in/radical-global-b6513691</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>MATRIX INFOTECH - Billing Accounting Inventory Software in Nagpur Reckon ERP</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>https://matrixsoftware.in/</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>+91 95952 76596</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>930, Central Ave, behind Kalra Petrol Pump, Chhota Loharpura, Gandhibagh, Nagpur, Maharashtra 440018, India</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>4.8</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>Not Available</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>https://in.linkedin.com/company/reckon-software-pvt-ltd</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Contiguvenzaa Private Limited</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>https://www.contiguvenzaa.com/</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>+91 84465 03094</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>72, Ekakshara, 1st floor, near jerryl lawn, Surendra Nagar, Vivekanand Nagar, Nagpur, Maharashtra 440015, India</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>3.8</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Not Acceptable!</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>Swapnil Zoad|https://in.linkedin.com/in/swapnil-zoad</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>https://in.linkedin.com/company/contiguvenzaa</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>https://in.linkedin.com/in/prayer-arje-843141237</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>ASW TECHNOLOGIES PVT. LTD.</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>https://www.aswtech.in/</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>+91 93706 71697</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>FLAT NO. 105, WING NO 01, RAJAT SANKUL, Ganeshpeth Colony, Nagpur, Maharashtra 440018, India</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>4.7</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>aswtech.in | 520: Web server is returning an unknown error</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>Sneha Kolte|https://in.linkedin.com/in/sneha-kolte-66a6bb254</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>https://in.linkedin.com/company/asw-technologies-pvt-ltd</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>https://in.linkedin.com/in/abhay-wagadre-544017a9</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Nice Software Solutions Pvt Ltd</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>http://www.nicesoftwaresolutions.com/</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>+91 80078 61579</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Plot No. 21, IT Park Rd, Gayatri Nagar, Pratap Nagar, Nagpur, Maharashtra 440022, India</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>4.1</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Get expert Data Analytics Services from a Top AI Consulting Company. As one of the Best AI Consulting Firms, we drive smarter decisions and business growth. Call us.</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>info@nicesoftwaresolutions.com</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>ADITYA SARAF|https://in.linkedin.com/in/aditya-saraf-0b36347</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>https://in.linkedin.com/company/nice-software-solutions</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Infinity Technology - Hospital Software, Clinic EMR &amp; IVF Software</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>http://www.infinitytechnology.in/</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>+91 88064 45533</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Vaishnav's Inn, Information Technology Park, 401, Sambhaji Nagar, Bhamti, Subhash Nagar, Sq, Nagpur, Maharashtra 440022, India</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>4.8</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Infinity Technology for Hospital Software </t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>infinitynagpur@gmail.com</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>Ajay Chaudhary|https://in.linkedin.com/in/ajay-chaudhary-80623196</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/infinity-healthcare-technology-solutions</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>https://in.linkedin.com/in/ajay-chaudhary-80623196</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Royals Webtech | Software Development, Website Developments, Mobile Application</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>https://www.royalswebtechpvtltd.com/</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>+91 87884 47944</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>4th floor, A Wing, Block No. 8, Mangalwari Complex, near Government Polytechnic, Sadar, Nagpur, Maharashtra 440001, India</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>4.3</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Royals Webtech: Software Company &amp; Digital Marketing in Nagpur, Mumbai India | Home</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>contact@royalswebtechpvtltd.com</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>Er. Chetan Wanjari|https://in.linkedin.com/in/chetanwanjari</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>https://in.linkedin.com/company/royalswebtech</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>https://in.linkedin.com/in/reena-singh-088125184</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J21"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Company</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Website</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Phone</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Address</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Rating</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Email</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>CEO</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Company LinkedIn</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>Leadership LinkedIn</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Abhi Engineering Corporation Pvt Ltd</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>http://abhiengineering.com//</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>+91 712 663 2808</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>404,405, law college square, W High Ct Rd, Master Colony, Tilak Nagar, Gokulpeth, Nagpur, Maharashtra 440010, India</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>4.5</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr"/>
+      <c r="G2" t="inlineStr"/>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>bhim Nidwancha|https://in.linkedin.com/in/bhim-nidwancha-2bb79236</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr"/>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>https://in.linkedin.com/in/rajesh-vishwkarma-00ba67152</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Paramount Engineering Company MIDC Nagpur</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>http://www.paramountengg.com/</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>+91 7104 329 262</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>42W4+53J, Wadi, Nagpur, Maharashtra 440016, India</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>4.7</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Not Acceptable!</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr"/>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>ROHIT TAPADIA|https://in.linkedin.com/in/rohit-tapadia-ba875a27</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>https://my.linkedin.com/company/paramount-engineering</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>https://in.linkedin.com/in/chetan-sontakke-65152665</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Central India Engineering Pvt Ltd</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>+91 73501 33335</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>F39 Tatya Tope Nagar, WHC Road, near Sai Catering Bichhayat Decorations, Maharashtra 440015, India</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>4.7</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr"/>
+      <c r="G4" t="inlineStr"/>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Jatin D. Rathi|https://in.linkedin.com/in/jatin-d-rathi-4a06a062</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr"/>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>https://in.linkedin.com/in/jatin-d-rathi-4a06a062</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Atlantis Engineers</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>http://atlantisengineers.com/</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>+91 98236 25317</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Little Flowers Nursery School, 172, Mohan Nagar, Nagpur, Maharashtra 440001, India</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>4.3</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Not Acceptable!</t>
+        </is>
+      </c>
       <c r="G5" t="inlineStr"/>
       <c r="H5" t="inlineStr">
         <is>
-          <t>Yogesh Kedar|https://in.linkedin.com/in/yogesh-kedar-65210734</t>
+          <t>George Efremidis|https://gr.linkedin.com/in/george-efremidis-3a80a05</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>https://in.linkedin.com/company/ocean-software-technologies</t>
-        </is>
-      </c>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>https://in.linkedin.com/in/yogesh-kedar-65210734</t>
-        </is>
-      </c>
+          <t>https://www.linkedin.com/company/atlantisengineering/</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Santosh Selokar Information Technology Pvt.Ltd Nagpur (SSIT.Pvt.Ltd)</t>
+          <t>Techture</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>https://www.ssinfotech.org/</t>
+          <t>http://www.techture.global/</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>+91 96579 59184</t>
+          <t>+91 91300 92843</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>FCI Housing Society, Plot no 9, Narendra Nagar Extension, New Narendra Nagar, Manish Nagar, Somalwada, Nagpur, Maharashtra 440015, India</t>
+          <t>30, behind Kotak Mahindra Bank, Shankar Nagar, East Shankar Nagar, Nagpur, Maharashtra 440010, India</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>4.6</t>
+          <t>4.1</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>SSIT</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr"/>
+          <t>Techture offers advanced VDC &amp; BIM services for design, planning, and construction efficiency. Drive accuracy and collaboration. Connect with us today!</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>contact@techture.global</t>
+        </is>
+      </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>santosh selokar|https://in.linkedin.com/in/santosh-selokar-4a62b831</t>
-        </is>
-      </c>
-      <c r="I6" t="inlineStr"/>
+          <t>Muhammad Zubair Khan|https://www.linkedin.com/in/zubairkh</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/techturestructures</t>
+        </is>
+      </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>https://in.linkedin.com/in/santosh-selokar-b7655618</t>
+          <t>https://www.linkedin.com/in/arnavjain92</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>GrowNixt Technologies Pvt. Ltd.</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr"/>
+          <t>SD ENGINEERING</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>http://sdstonesengineering.com/</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>+91 84593 16306</t>
+        </is>
+      </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>IT Park Nagpur IT Park road Gayatri appartment 202, Nagpur, Maharashtra 440022, India</t>
+          <t>Flat No 104 Tulip Apartment Ram Krishna Nagari New Narsara Road Opp Indian, Gas Godown, Nagpur, Maharashtra 440034, India</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>4.9</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr"/>
+          <t>4.8</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>SD Engineering</t>
+        </is>
+      </c>
       <c r="G7" t="inlineStr"/>
       <c r="H7" t="inlineStr">
         <is>
-          <t>rewan gadkari|https://in.linkedin.com/in/rewan-gadkari-883804225</t>
+          <t>Baasansuren Boris|https://mn.linkedin.com/in/baasansuren-boris-4561a214</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>https://in.linkedin.com/company/grownixt-technologies</t>
-        </is>
-      </c>
-      <c r="J7" t="inlineStr">
-        <is>
-          <t>https://in.linkedin.com/in/rewan-gadkari-883804225</t>
-        </is>
-      </c>
+          <t>https://www.linkedin.com/company/sdengineering</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>S R solutions</t>
+          <t>Shree Om Sai Construction Nitishka Pvt Ltd - Building Construction</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>https://digitronsoftwares.com/</t>
+          <t>https://soscnpltd.in/</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>+91 77092 66577</t>
+          <t>+91 91752 66870</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>2nd FLOOR, 10A, c/o, Main Rd, above SAI ENTERPRIESE, beside CANARA ATM, New Diamond Nagar, Shaktimata Nagar, Nandanvan, Nagpur, Maharashtra 440024, India</t>
+          <t>plot no 402, opposite Jaswant tuli mall, Near Indora Chowk, Model Town, Nagpur, Maharashtra 440014, India</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -778,210 +1759,188 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>this is multilingual example meta tag for english</t>
+          <t>soscnpltd</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>digitronsoftwares@gmail.com</t>
+          <t>info@soscnpltd.in</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>Tessy Anifowoshe sr|https://www.linkedin.com/in/tessy-anifowoshe-sr-9a135a184</t>
-        </is>
-      </c>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>https://in.linkedin.com/company/sr-solutions-realesateservices</t>
-        </is>
-      </c>
+          <t>Amitesh Arun|https://in.linkedin.com/in/amitesh-arun-007386121</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr"/>
       <c r="J8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Pixel Values Technolabs | Software Company</t>
+          <t>BHORE ENGINEERING CONSULTANTS PVT. LTD.</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>https://www.pixelvalues.com/</t>
+          <t>https://bhoreengineering.com/</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>+91 84848 36319</t>
+          <t>+91 93212 35472</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Swapna Apartment, 35, beside Mantri Sadan, Shivaji Nagar, Nagpur, Maharashtra 440010, India</t>
+          <t>38, Khamla Rd, Near Tajshree Honda, Ramakrishna Nagar, Vivekanand Nagar, Nagpur, Maharashtra 440015, India</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>4.8</t>
+          <t>4.7</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Pixel Values is a Best Mobile App Development Company and among the Top Web Development Companies offering custom Android, iOS, and scalable web solutions.</t>
+          <t>Bhore Engineering Consultants – BEC</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>info@pixelvalues.com</t>
+          <t>cvbhore@gmail.com</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>Tauseef Anwar|https://in.linkedin.com/in/tauseefanwar</t>
+          <t>Dr. Chaitanya V. Bhore|https://in.linkedin.com/in/chaitanyavbhore</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/pixel-values-techno-labs</t>
+          <t>https://in.linkedin.com/company/bhore-engineering-consultants-pvt-ltd</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>https://in.linkedin.com/in/tauseefanwar</t>
+          <t>https://in.linkedin.com/in/chaitanyavbhore</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Xceller IT Services</t>
+          <t>OneClick BIM Private Limited</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>http://www.xceller.com/</t>
+          <t>http://www.oneclickbim.global/</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>+91 93267 44884</t>
+          <t>+91 87889 46040</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>13/1, Diglin Industries, IT Park Rd, Parsodi, Nagpur, Maharashtra 440022, India</t>
+          <t>Basant Apartment, 201, Kadbi Square, Clark Town, Nagpur, Maharashtra 440014, India</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>4.5</t>
+          <t>4.8</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Discover tailored IT services &amp; solutions at Xceller. From consulting to development, we empower your business with reliable tech expertise and innovation.</t>
-        </is>
-      </c>
-      <c r="G10" t="inlineStr"/>
+          <t>Oneclick BIM is Engineering Consultants offers BIM Services, including architectural, structural, civil, CAD, BIM, detailing, and, electrical.</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>abhijeet@oneclickbim.global</t>
+        </is>
+      </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>Anshu S|https://in.linkedin.com/in/anshu-s-74bb41217</t>
+          <t>ABHIJEET P|https://in.linkedin.com/in/abhijeet-ocb</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>https://au.linkedin.com/company/xcellerate-it</t>
-        </is>
-      </c>
-      <c r="J10" t="inlineStr">
-        <is>
-          <t>https://in.linkedin.com/in/mohit-lanjewar-9199a5294</t>
-        </is>
-      </c>
+          <t>https://in.linkedin.com/company/one-click-bim-cad-services-company-india-dubai</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Callisto IT Solutions - Best Software Development , Web Application Development and Training &amp; IT InternshipCompany</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>http://www.callistoitsolutions.com/</t>
+          <t>Dhansa Architect and Engineering Consultant</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>+91 70572 05423</t>
+          <t>+91 80552 19446</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>4 - Shivshakti App, Bhagwan Nagar Rd, Banarjee Layout, Rameshwari, Nagpur, Maharashtra 440027, India</t>
+          <t>1ST FLOOR, CHATRAPATI SQUARE, PLOT NO 50, RING ROAD, Gawande layout, Khamla, Nagpur, Maharashtra 440015, India</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>4.4</t>
+          <t>4.9</t>
         </is>
       </c>
       <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr"/>
       <c r="H11" t="inlineStr">
         <is>
-          <t>Not Available</t>
-        </is>
-      </c>
-      <c r="I11" t="inlineStr">
-        <is>
-          <t>https://in.linkedin.com/company/callisto-it-solutions</t>
-        </is>
-      </c>
-      <c r="J11" t="inlineStr"/>
+          <t>Dhansa Architect|https://in.linkedin.com/in/dhansa-architect-047042237</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr"/>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>https://in.linkedin.com/in/aditya-bhakte-a3b373153</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Nass Technologies - Software Development &amp; IT Training</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>http://www.nasstechnologies.com/</t>
+          <t>Rosmith Engineering</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>+91 82372 66913</t>
+          <t>+91 94049 02636</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>1st Floor, 13, Plot No 5, Borgaon Rd, beside HDFC Bank, near Jafar Nagar, Sugat Colony, Jafar Nagar, Police Line Takli, Nagpur, Maharashtra 440013, India</t>
+          <t>185, Vedant, Dixit Nagar, Nagpur, Maharashtra 440026, India</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>4.6</t>
-        </is>
-      </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>Nass Technologies has the most advanced digital solutions for your organisation. Web development and mobile apps are the first steps in digital transformation.</t>
-        </is>
-      </c>
-      <c r="G12" t="inlineStr">
-        <is>
-          <t>info@nasstechnologies.com</t>
-        </is>
-      </c>
+          <t>4.8</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr"/>
+      <c r="G12" t="inlineStr"/>
       <c r="H12" t="inlineStr">
         <is>
-          <t>Valivullah Michael|https://www.linkedin.com/in/valivullah-michael-1b337471</t>
+          <t>Richard Smith Jr|https://www.linkedin.com/in/richard-smith-jr-041a611a3</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>https://in.linkedin.com/company/nass-technologies</t>
+          <t>https://www.linkedin.com/company/rasmith</t>
         </is>
       </c>
       <c r="J12" t="inlineStr"/>
@@ -989,438 +1948,408 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>TALLYTACT LLP</t>
+          <t>imaGIS Engineering Solutions Pvt. Ltd</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>https://www.tallytact.com/</t>
+          <t>http://www.imagis.co.in/</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>+91 93266 47411</t>
+          <t>+91 712 222 2137</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Plot no.80, opp. Nirman Enclave, Gajanan Nagar, Nagpur, Maharashtra 440015, India</t>
+          <t>Plot No. 13, 2, IT Park Rd, near Gayatri Nagar, Subhash Nagar, Pratap Nagar, Nagpur, Maharashtra 440022, India</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>4.8</t>
-        </is>
-      </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>TALLYTACT LLP is helping Accountant &amp; CAs solving all TallyPrime Release 7.0 related all problems.</t>
-        </is>
-      </c>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>sales@tallytact.com</t>
-        </is>
-      </c>
+          <t>4.6</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr"/>
+      <c r="G13" t="inlineStr"/>
       <c r="H13" t="inlineStr">
         <is>
-          <t>Not Available</t>
+          <t>Sandeep Shirkhedkar|https://in.linkedin.com/in/sandeep-shirkhedkar-b0271040</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>https://in.linkedin.com/company/tallytact-llp</t>
+          <t>https://in.linkedin.com/company/imagis-engineering-solutions</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>https://in.linkedin.com/in/mayur-tajnekar</t>
+          <t>https://in.linkedin.com/in/imagis-engineering-solutions-private-limited-nagpur-a9273a358</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Pegasus Technologies &amp; Software Private Limited Best Data Science analytics institute In Nagpur</t>
+          <t>Sanghi Consulting Engineers India Pvt. Ltd</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>http://pegasusacademy.in/</t>
+          <t>http://sanghigroup.org/</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>+91 98235 20987</t>
+          <t>+91 712 224 9225</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Plot No. 43, Mire Layout, Kabir Nagar, Nandanvan, Nagpur, Maharashtra 440009, India</t>
+          <t>101, Laxmi Keshav Apartments, near Park corner, Dhantoli, Nagpur, Maharashtra 440012, India</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>4.5</t>
-        </is>
-      </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>Pegasus Academy – Training | Certification | Placement</t>
-        </is>
-      </c>
-      <c r="G14" t="inlineStr"/>
+          <t>3.9</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr"/>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>user@domain.com</t>
+        </is>
+      </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>Not Available</t>
+          <t>Rohit Francis|https://in.linkedin.com/in/rohit-francis-b12385183</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>https://in.linkedin.com/company/pegasus-technologies-software-pvt-ltd</t>
+          <t>https://in.linkedin.com/company/sanghi-consulting-engineers-india-pvt-ltd-</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>https://in.linkedin.com/in/komal-tembhare-21b700236</t>
+          <t>https://in.linkedin.com/in/rohit-francis-b12385183</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Radical Global</t>
+          <t>PEB BlueLadder EPC Solutions Pvt Ltd | Pre Engineered Building Solutions | PEB Structure Manufacturer In Nagpur</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>http://www.radicalglobal.net/</t>
+          <t>http://www.blueladderepc.com/</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>+91 90212 51392</t>
+          <t>+91 77988 11367</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>1, Besides Deendayal Uppadhaya Garden, 94, Jawahar Nagar, Raghuji Nagar, Nagpur, Maharashtra 440024, India</t>
+          <t>6th Floor, Landmark building, Ramdaspeth, Nagpur, Maharashtra 440010, India</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>4.8</t>
+          <t>4.1</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Radical Global – Digital Workplace Services</t>
+          <t>Leading PEB manufacturer and EPC solution provider in India. Industrial sheds, warehouses, and turnkey construction services.</t>
         </is>
       </c>
       <c r="G15" t="inlineStr"/>
       <c r="H15" t="inlineStr">
         <is>
-          <t>Vibhor Khatwar|https://in.linkedin.com/in/vibhor-khatwar-6870485b</t>
+          <t>Sagar Kewalramani|https://in.linkedin.com/in/sagar-kewalramani-1a0979155</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>https://in.linkedin.com/company/radicalglobalcompany</t>
+          <t>https://in.linkedin.com/company/blueladder-epc-solutions</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>https://in.linkedin.com/in/radical-global-b6513691</t>
+          <t>https://in.linkedin.com/in/sagar-kewalramani-1a0979155</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>MATRIX INFOTECH - Billing Accounting Inventory Software in Nagpur Reckon ERP</t>
+          <t>Patankar Consultants Pvt. Ltd</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>https://matrixsoftware.in/</t>
+          <t>http://www.patankarconsultants.com/</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>+91 95952 76596</t>
+          <t>+91 712 224 9293</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>930, Central Ave, behind Kalra Petrol Pump, Chhota Loharpura, Gandhibagh, Nagpur, Maharashtra 440018, India</t>
+          <t>79, Universal Annex,, Shivaji Nagar, Nagpur, Maharashtra 440010, India</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>4.8</t>
+          <t>4.6</t>
         </is>
       </c>
       <c r="F16" t="inlineStr"/>
-      <c r="G16" t="inlineStr"/>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>project@patankarconsultants.com</t>
+        </is>
+      </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>Not Available</t>
+          <t>P S Patankar|https://in.linkedin.com/in/p-s-patankar-1576a764</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>https://in.linkedin.com/company/reckon-software-pvt-ltd</t>
-        </is>
-      </c>
-      <c r="J16" t="inlineStr"/>
+          <t>https://in.linkedin.com/company/patankar-consultants-pvt-ltd</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>https://in.linkedin.com/in/p-s-patankar-1576a764</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Contiguvenzaa Private Limited</t>
+          <t>Divya Consultants</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>https://www.contiguvenzaa.com/</t>
+          <t>http://divyaconsultants.in/</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>+91 84465 03094</t>
+          <t>+91 712 276 6143</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>72, Ekakshara, 1st floor, near jerryl lawn, Surendra Nagar, Vivekanand Nagar, Nagpur, Maharashtra 440015, India</t>
+          <t>303, Aarna Complex, Darodkar Square, Central Ave, Ladpura, Itwari, Nagpur, Maharashtra 440002, India</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>3.8</t>
-        </is>
-      </c>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>Not Acceptable!</t>
-        </is>
-      </c>
-      <c r="G17" t="inlineStr"/>
+          <t>4.9</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr"/>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>design@divya-consultants.com</t>
+        </is>
+      </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>Swapnil Zoad|https://in.linkedin.com/in/swapnil-zoad</t>
+          <t>Divya Gupta|https://www.linkedin.com/in/gridsconsulting</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>https://in.linkedin.com/company/contiguvenzaa</t>
+          <t>https://in.linkedin.com/company/divya-consultants</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>https://in.linkedin.com/in/prayer-arje-843141237</t>
+          <t>https://in.linkedin.com/in/divya-chavan-bb2142118</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>ASW TECHNOLOGIES PVT. LTD.</t>
+          <t>Vishwa MEP Engineers Pvt.Ltd</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>https://www.aswtech.in/</t>
+          <t>https://vishwa.co/</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>+91 93706 71697</t>
+          <t>+91 712 660 6535</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>FLAT NO. 105, WING NO 01, RAJAT SANKUL, Ganeshpeth Colony, Nagpur, Maharashtra 440018, India</t>
+          <t>43W4+R6P, Ravinagar Square, Yashwant Nagar, Nagpur, Maharashtra 440033, India</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>4.7</t>
-        </is>
-      </c>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>aswtech.in | 520: Web server is returning an unknown error</t>
-        </is>
-      </c>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr"/>
       <c r="G18" t="inlineStr"/>
       <c r="H18" t="inlineStr">
         <is>
-          <t>Sneha Kolte|https://in.linkedin.com/in/sneha-kolte-66a6bb254</t>
-        </is>
-      </c>
-      <c r="I18" t="inlineStr">
-        <is>
-          <t>https://in.linkedin.com/company/asw-technologies-pvt-ltd</t>
-        </is>
-      </c>
+          <t>Kishor Choudhari|https://in.linkedin.com/in/kishor-choudhari-a3a59063</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr"/>
       <c r="J18" t="inlineStr">
         <is>
-          <t>https://in.linkedin.com/in/abhay-wagadre-544017a9</t>
+          <t>https://in.linkedin.com/in/kishor-choudhari-a3a59063</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Nice Software Solutions Pvt Ltd</t>
+          <t>Ahmad Construction &amp; Interiors</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>http://www.nicesoftwaresolutions.com/</t>
+          <t>https://www.instagram.com/ahmad_construction_interiors?igsh=enR0YTFmampnczRw</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>+91 80078 61579</t>
+          <t>+91 76209 28833</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Plot No. 21, IT Park Rd, Gayatri Nagar, Pratap Nagar, Nagpur, Maharashtra 440022, India</t>
+          <t>102, Aman's Villa, Eidgh Ground, above Shahu Kirana, Adarsh Colony, Jafar Nagar, New Mankapur, Nagpur, Maharashtra 440013, India</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>4.1</t>
+          <t>4.9</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Get expert Data Analytics Services from a Top AI Consulting Company. As one of the Best AI Consulting Firms, we drive smarter decisions and business growth. Call us.</t>
-        </is>
-      </c>
-      <c r="G19" t="inlineStr">
-        <is>
-          <t>info@nicesoftwaresolutions.com</t>
-        </is>
-      </c>
+          <t>384 Followers, 1,096 Following, 40 Posts - Osman Furniture &amp; Interior (@ahmad_construction_interiors) on Instagram: "Contact Us:-7620928833
+Building Construction,⚒️
+Interior Design
+Modular Furniture
+Civil Engg Drawing🏙️
+Architectural Planning💻 
+3d View
+Nagpur"</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr"/>
       <c r="H19" t="inlineStr">
         <is>
-          <t>ADITYA SARAF|https://in.linkedin.com/in/aditya-saraf-0b36347</t>
+          <t>Junaid Ahmed|https://in.linkedin.com/in/junaid-ahmed-0283082b4</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>https://in.linkedin.com/company/nice-software-solutions</t>
-        </is>
-      </c>
-      <c r="J19" t="inlineStr"/>
+          <t>https://pk.linkedin.com/company/accopakistan</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>https://in.linkedin.com/in/afzaal-ahmad-136044307</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Infinity Technology - Hospital Software, Clinic EMR &amp; IVF Software</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>http://www.infinitytechnology.in/</t>
+          <t>DUSON CIVIL ENGINEERING SERVICES LLP</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>+91 88064 45533</t>
+          <t>+91 712 224 3354</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Vaishnav's Inn, Information Technology Park, 401, Sambhaji Nagar, Bhamti, Subhash Nagar, Sq, Nagpur, Maharashtra 440022, India</t>
+          <t>35, Khamla Rd, Deo Nagar, Nagpur, Maharashtra 440015, India</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>4.8</t>
-        </is>
-      </c>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Infinity Technology for Hospital Software </t>
-        </is>
-      </c>
-      <c r="G20" t="inlineStr">
-        <is>
-          <t>infinitynagpur@gmail.com</t>
-        </is>
-      </c>
+          <t>4.5</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr"/>
+      <c r="G20" t="inlineStr"/>
       <c r="H20" t="inlineStr">
         <is>
-          <t>Ajay Chaudhary|https://in.linkedin.com/in/ajay-chaudhary-80623196</t>
-        </is>
-      </c>
-      <c r="I20" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/company/infinity-healthcare-technology-solutions</t>
-        </is>
-      </c>
+          <t>Arpit Veldi|https://in.linkedin.com/in/arpit-veldi-573a15a8</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr"/>
       <c r="J20" t="inlineStr">
         <is>
-          <t>https://in.linkedin.com/in/ajay-chaudhary-80623196</t>
+          <t>https://in.linkedin.com/in/sangharshal</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Royals Webtech | Software Development, Website Developments, Mobile Application</t>
+          <t>Mann Engineering Company</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>https://www.royalswebtechpvtltd.com/</t>
+          <t>http://mannengineeringcompany.com/</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>+91 87884 47944</t>
+          <t>+91 99227 00037</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>4th floor, A Wing, Block No. 8, Mangalwari Complex, near Government Polytechnic, Sadar, Nagpur, Maharashtra 440001, India</t>
+          <t>Kamptee Rd, Pili Nadi, Nagpur, Maharashtra 440026, India</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>4.3</t>
-        </is>
-      </c>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>Royals Webtech: Software Company &amp; Digital Marketing in Nagpur, Mumbai India | Home</t>
-        </is>
-      </c>
-      <c r="G21" t="inlineStr">
-        <is>
-          <t>contact@royalswebtechpvtltd.com</t>
-        </is>
-      </c>
+          <t>4.6</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr"/>
+      <c r="G21" t="inlineStr"/>
       <c r="H21" t="inlineStr">
         <is>
-          <t>Er. Chetan Wanjari|https://in.linkedin.com/in/chetanwanjari</t>
+          <t>Steve Mann|https://www.linkedin.com/in/steve-mann-71971041</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>https://in.linkedin.com/company/royalswebtech</t>
-        </is>
-      </c>
-      <c r="J21" t="inlineStr">
-        <is>
-          <t>https://in.linkedin.com/in/reena-singh-088125184</t>
-        </is>
-      </c>
+          <t>https://ie.linkedin.com/company/mann-engineering</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Create add new project button
</commit_message>
<xml_diff>
--- a/company_leads.xlsx
+++ b/company_leads.xlsx
@@ -10,6 +10,7 @@
     <sheet name="Sheet" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="CodePilot AI" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="chatbot outlook ai" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Chatbot AI" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -2385,4 +2386,70 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Company</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Website</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Phone</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Address</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Rating</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Email</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>CEO</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Company LinkedIn</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>Leadership LinkedIn</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Added the overview button at the sidebar
</commit_message>
<xml_diff>
--- a/company_leads.xlsx
+++ b/company_leads.xlsx
@@ -11,6 +11,8 @@
     <sheet name="CodePilot AI" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="chatbot outlook ai" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Chatbot AI" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="chatbot outlook ai1" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Chatbot AI1" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -2452,4 +2454,136 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Company</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Website</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Phone</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Address</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Rating</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Email</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>CEO</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Company LinkedIn</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>Leadership LinkedIn</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Company</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Website</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Phone</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Address</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Rating</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Email</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>CEO</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Company LinkedIn</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>Leadership LinkedIn</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Fixed the sidebar and added logo in overview
</commit_message>
<xml_diff>
--- a/company_leads.xlsx
+++ b/company_leads.xlsx
@@ -13,6 +13,8 @@
     <sheet name="Chatbot AI" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="chatbot outlook ai1" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="Chatbot AI1" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="hello" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="CodePilot AI1" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -2586,4 +2588,1019 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Company</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Website</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Phone</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Address</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Rating</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Email</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>CEO</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Company LinkedIn</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>Leadership LinkedIn</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J21"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Company</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Website</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Phone</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Address</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Rating</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Email</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>CEO</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Company LinkedIn</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>Leadership LinkedIn</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Abhi Engineering Corporation Pvt Ltd</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>http://abhiengineering.com//</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>+91 712 663 2808</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>404,405, law college square, W High Ct Rd, Master Colony, Tilak Nagar, Gokulpeth, Nagpur, Maharashtra 440010, India</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>4.5</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr"/>
+      <c r="G2" t="inlineStr"/>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>bhim Nidwancha|https://in.linkedin.com/in/bhim-nidwancha-2bb79236</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr"/>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>https://in.linkedin.com/in/rajesh-vishwkarma-00ba67152</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Paramount Engineering Company MIDC Nagpur</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>http://www.paramountengg.com/</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>+91 7104 329 262</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>42W4+53J, Wadi, Nagpur, Maharashtra 440016, India</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>4.7</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Not Acceptable!</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr"/>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>ROHIT TAPADIA|https://in.linkedin.com/in/rohit-tapadia-ba875a27</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>https://my.linkedin.com/company/paramount-engineering</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>https://in.linkedin.com/in/chetan-sontakke-65152665</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Central India Engineering Pvt Ltd</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>+91 73501 33335</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>F39 Tatya Tope Nagar, WHC Road, near Sai Catering Bichhayat Decorations, Maharashtra 440015, India</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>4.7</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr"/>
+      <c r="G4" t="inlineStr"/>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Jatin D. Rathi|https://in.linkedin.com/in/jatin-d-rathi-4a06a062</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr"/>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>https://in.linkedin.com/in/jatin-d-rathi-4a06a062</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Atlantis Engineers</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>http://atlantisengineers.com/</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>+91 98236 25317</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Little Flowers Nursery School, 172, Mohan Nagar, Nagpur, Maharashtra 440001, India</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>4.3</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Not Acceptable!</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr"/>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>George Efremidis|https://gr.linkedin.com/in/george-efremidis-3a80a05</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/atlantisengineering/</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Techture</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>http://www.techture.global/</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>+91 91300 92843</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>30, behind Kotak Mahindra Bank, Shankar Nagar, East Shankar Nagar, Nagpur, Maharashtra 440010, India</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>4.1</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Techture offers advanced VDC &amp; BIM services for design, planning, and construction efficiency. Drive accuracy and collaboration. Connect with us today!</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>contact@techture.global</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Muhammad Zubair Khan|https://www.linkedin.com/in/zubairkh</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/techturestructures</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/arnavjain92</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>SD ENGINEERING</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>http://sdstonesengineering.com/</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>+91 84593 16306</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Flat No 104 Tulip Apartment Ram Krishna Nagari New Narsara Road Opp Indian, Gas Godown, Nagpur, Maharashtra 440034, India</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>4.8</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>SD Engineering</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr"/>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Baasansuren Boris|https://mn.linkedin.com/in/baasansuren-boris-4561a214</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/sdengineering</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Shree Om Sai Construction Nitishka Pvt Ltd - Building Construction</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>https://soscnpltd.in/</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>+91 91752 66870</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>plot no 402, opposite Jaswant tuli mall, Near Indora Chowk, Model Town, Nagpur, Maharashtra 440014, India</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>4.7</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>soscnpltd</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>info@soscnpltd.in</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Amitesh Arun|https://in.linkedin.com/in/amitesh-arun-007386121</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr"/>
+      <c r="J8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>BHORE ENGINEERING CONSULTANTS PVT. LTD.</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>https://bhoreengineering.com/</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>+91 93212 35472</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>38, Khamla Rd, Near Tajshree Honda, Ramakrishna Nagar, Vivekanand Nagar, Nagpur, Maharashtra 440015, India</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>4.7</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Bhore Engineering Consultants – BEC</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>cvbhore@gmail.com</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Dr. Chaitanya V. Bhore|https://in.linkedin.com/in/chaitanyavbhore</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>https://in.linkedin.com/company/bhore-engineering-consultants-pvt-ltd</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>https://in.linkedin.com/in/chaitanyavbhore</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>OneClick BIM Private Limited</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>http://www.oneclickbim.global/</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>+91 87889 46040</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Basant Apartment, 201, Kadbi Square, Clark Town, Nagpur, Maharashtra 440014, India</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>4.8</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Oneclick BIM is Engineering Consultants offers BIM Services, including architectural, structural, civil, CAD, BIM, detailing, and, electrical.</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>abhijeet@oneclickbim.global</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>ABHIJEET P|https://in.linkedin.com/in/abhijeet-ocb</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>https://in.linkedin.com/company/one-click-bim-cad-services-company-india-dubai</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Dhansa Architect and Engineering Consultant</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>+91 80552 19446</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>1ST FLOOR, CHATRAPATI SQUARE, PLOT NO 50, RING ROAD, Gawande layout, Khamla, Nagpur, Maharashtra 440015, India</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>4.9</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr"/>
+      <c r="G11" t="inlineStr"/>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Dhansa Architect|https://in.linkedin.com/in/dhansa-architect-047042237</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr"/>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>https://in.linkedin.com/in/aditya-bhakte-a3b373153</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Rosmith Engineering</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>+91 94049 02636</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>185, Vedant, Dixit Nagar, Nagpur, Maharashtra 440026, India</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>4.8</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr"/>
+      <c r="G12" t="inlineStr"/>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Richard Smith Jr|https://www.linkedin.com/in/richard-smith-jr-041a611a3</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/rasmith</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>imaGIS Engineering Solutions Pvt. Ltd</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>http://www.imagis.co.in/</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>+91 712 222 2137</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Plot No. 13, 2, IT Park Rd, near Gayatri Nagar, Subhash Nagar, Pratap Nagar, Nagpur, Maharashtra 440022, India</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>4.6</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr"/>
+      <c r="G13" t="inlineStr"/>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Sandeep Shirkhedkar|https://in.linkedin.com/in/sandeep-shirkhedkar-b0271040</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>https://in.linkedin.com/company/imagis-engineering-solutions</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>https://in.linkedin.com/in/imagis-engineering-solutions-private-limited-nagpur-a9273a358</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Sanghi Consulting Engineers India Pvt. Ltd</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>http://sanghigroup.org/</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>+91 712 224 9225</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>101, Laxmi Keshav Apartments, near Park corner, Dhantoli, Nagpur, Maharashtra 440012, India</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>3.9</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr"/>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>user@domain.com</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>Rohit Francis|https://in.linkedin.com/in/rohit-francis-b12385183</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>https://in.linkedin.com/company/sanghi-consulting-engineers-india-pvt-ltd-</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>https://in.linkedin.com/in/rohit-francis-b12385183</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>PEB BlueLadder EPC Solutions Pvt Ltd | Pre Engineered Building Solutions | PEB Structure Manufacturer In Nagpur</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>http://www.blueladderepc.com/</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>+91 77988 11367</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>6th Floor, Landmark building, Ramdaspeth, Nagpur, Maharashtra 440010, India</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>4.1</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Leading PEB manufacturer and EPC solution provider in India. Industrial sheds, warehouses, and turnkey construction services.</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr"/>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Sagar Kewalramani|https://in.linkedin.com/in/sagar-kewalramani-1a0979155</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>https://in.linkedin.com/company/blueladder-epc-solutions</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>https://in.linkedin.com/in/sagar-kewalramani-1a0979155</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Patankar Consultants Pvt. Ltd</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>http://www.patankarconsultants.com/</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>+91 712 224 9293</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>79, Universal Annex,, Shivaji Nagar, Nagpur, Maharashtra 440010, India</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>4.6</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr"/>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>project@patankarconsultants.com</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>P S Patankar|https://in.linkedin.com/in/p-s-patankar-1576a764</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>https://in.linkedin.com/company/patankar-consultants-pvt-ltd</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>https://in.linkedin.com/in/p-s-patankar-1576a764</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Divya Consultants</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>http://divyaconsultants.in/</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>+91 712 276 6143</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>303, Aarna Complex, Darodkar Square, Central Ave, Ladpura, Itwari, Nagpur, Maharashtra 440002, India</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>4.9</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr"/>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>design@divya-consultants.com</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>Divya Gupta|https://www.linkedin.com/in/gridsconsulting</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>https://in.linkedin.com/company/divya-consultants</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>https://in.linkedin.com/in/divya-chavan-bb2142118</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Vishwa MEP Engineers Pvt.Ltd</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>https://vishwa.co/</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>+91 712 660 6535</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>43W4+R6P, Ravinagar Square, Yashwant Nagar, Nagpur, Maharashtra 440033, India</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr"/>
+      <c r="G18" t="inlineStr"/>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>Kishor Choudhari|https://in.linkedin.com/in/kishor-choudhari-a3a59063</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr"/>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>https://in.linkedin.com/in/kishor-choudhari-a3a59063</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Ahmad Construction &amp; Interiors</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/ahmad_construction_interiors?igsh=enR0YTFmampnczRw</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>+91 76209 28833</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>102, Aman's Villa, Eidgh Ground, above Shahu Kirana, Adarsh Colony, Jafar Nagar, New Mankapur, Nagpur, Maharashtra 440013, India</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>4.9</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>384 Followers, 1,096 Following, 40 Posts - Osman Furniture &amp; Interior (@ahmad_construction_interiors) on Instagram: "Contact Us:-7620928833
+Building Construction,⚒️
+Interior Design
+Modular Furniture
+Civil Engg Drawing🏙️
+Architectural Planning💻 
+3d View
+Nagpur"</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr"/>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>Junaid Ahmed|https://in.linkedin.com/in/junaid-ahmed-0283082b4</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>https://pk.linkedin.com/company/accopakistan</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>https://in.linkedin.com/in/afzaal-ahmad-136044307</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>DUSON CIVIL ENGINEERING SERVICES LLP</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>+91 712 224 3354</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>35, Khamla Rd, Deo Nagar, Nagpur, Maharashtra 440015, India</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>4.5</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr"/>
+      <c r="G20" t="inlineStr"/>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>Arpit Veldi|https://in.linkedin.com/in/arpit-veldi-573a15a8</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr"/>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>https://in.linkedin.com/in/sangharshal</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Mann Engineering Company</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>http://mannengineeringcompany.com/</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>+91 99227 00037</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Kamptee Rd, Pili Nadi, Nagpur, Maharashtra 440026, India</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>4.6</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr"/>
+      <c r="G21" t="inlineStr"/>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>Steve Mann|https://www.linkedin.com/in/steve-mann-71971041</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>https://ie.linkedin.com/company/mann-engineering</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Fixed the merge conflict issue
</commit_message>
<xml_diff>
--- a/company_leads.xlsx
+++ b/company_leads.xlsx
@@ -15,6 +15,8 @@
     <sheet name="Chatbot AI1" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="hello" sheetId="7" state="visible" r:id="rId7"/>
     <sheet name="CodePilot AI1" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="CodePilot AI2" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="gg" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1413,6 +1415,72 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Company</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Website</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Phone</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Address</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Rating</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Email</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>CEO</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Company LinkedIn</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>Leadership LinkedIn</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
@@ -2743,14 +2811,11 @@
           <t>4.5</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr"/>
-      <c r="G2" t="inlineStr"/>
       <c r="H2" t="inlineStr">
         <is>
           <t>bhim Nidwancha|https://in.linkedin.com/in/bhim-nidwancha-2bb79236</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr"/>
       <c r="J2" t="inlineStr">
         <is>
           <t>https://in.linkedin.com/in/rajesh-vishwkarma-00ba67152</t>
@@ -2788,7 +2853,6 @@
           <t>Not Acceptable!</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr"/>
       <c r="H3" t="inlineStr">
         <is>
           <t>ROHIT TAPADIA|https://in.linkedin.com/in/rohit-tapadia-ba875a27</t>
@@ -2826,14 +2890,11 @@
           <t>4.7</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr"/>
-      <c r="G4" t="inlineStr"/>
       <c r="H4" t="inlineStr">
         <is>
           <t>Jatin D. Rathi|https://in.linkedin.com/in/jatin-d-rathi-4a06a062</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr"/>
       <c r="J4" t="inlineStr">
         <is>
           <t>https://in.linkedin.com/in/jatin-d-rathi-4a06a062</t>
@@ -2871,7 +2932,6 @@
           <t>Not Acceptable!</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr"/>
       <c r="H5" t="inlineStr">
         <is>
           <t>George Efremidis|https://gr.linkedin.com/in/george-efremidis-3a80a05</t>
@@ -2882,7 +2942,6 @@
           <t>https://www.linkedin.com/company/atlantisengineering/</t>
         </is>
       </c>
-      <c r="J5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -2967,7 +3026,6 @@
           <t>SD Engineering</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr"/>
       <c r="H7" t="inlineStr">
         <is>
           <t>Baasansuren Boris|https://mn.linkedin.com/in/baasansuren-boris-4561a214</t>
@@ -2978,7 +3036,6 @@
           <t>https://www.linkedin.com/company/sdengineering</t>
         </is>
       </c>
-      <c r="J7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -3021,8 +3078,6 @@
           <t>Amitesh Arun|https://in.linkedin.com/in/amitesh-arun-007386121</t>
         </is>
       </c>
-      <c r="I8" t="inlineStr"/>
-      <c r="J8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -3122,7 +3177,6 @@
           <t>https://in.linkedin.com/company/one-click-bim-cad-services-company-india-dubai</t>
         </is>
       </c>
-      <c r="J10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -3145,14 +3199,11 @@
           <t>4.9</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr"/>
-      <c r="G11" t="inlineStr"/>
       <c r="H11" t="inlineStr">
         <is>
           <t>Dhansa Architect|https://in.linkedin.com/in/dhansa-architect-047042237</t>
         </is>
       </c>
-      <c r="I11" t="inlineStr"/>
       <c r="J11" t="inlineStr">
         <is>
           <t>https://in.linkedin.com/in/aditya-bhakte-a3b373153</t>
@@ -3180,8 +3231,6 @@
           <t>4.8</t>
         </is>
       </c>
-      <c r="F12" t="inlineStr"/>
-      <c r="G12" t="inlineStr"/>
       <c r="H12" t="inlineStr">
         <is>
           <t>Richard Smith Jr|https://www.linkedin.com/in/richard-smith-jr-041a611a3</t>
@@ -3192,7 +3241,6 @@
           <t>https://www.linkedin.com/company/rasmith</t>
         </is>
       </c>
-      <c r="J12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -3220,8 +3268,6 @@
           <t>4.6</t>
         </is>
       </c>
-      <c r="F13" t="inlineStr"/>
-      <c r="G13" t="inlineStr"/>
       <c r="H13" t="inlineStr">
         <is>
           <t>Sandeep Shirkhedkar|https://in.linkedin.com/in/sandeep-shirkhedkar-b0271040</t>
@@ -3264,7 +3310,6 @@
           <t>3.9</t>
         </is>
       </c>
-      <c r="F14" t="inlineStr"/>
       <c r="G14" t="inlineStr">
         <is>
           <t>user@domain.com</t>
@@ -3317,7 +3362,6 @@
           <t>Leading PEB manufacturer and EPC solution provider in India. Industrial sheds, warehouses, and turnkey construction services.</t>
         </is>
       </c>
-      <c r="G15" t="inlineStr"/>
       <c r="H15" t="inlineStr">
         <is>
           <t>Sagar Kewalramani|https://in.linkedin.com/in/sagar-kewalramani-1a0979155</t>
@@ -3360,7 +3404,6 @@
           <t>4.6</t>
         </is>
       </c>
-      <c r="F16" t="inlineStr"/>
       <c r="G16" t="inlineStr">
         <is>
           <t>project@patankarconsultants.com</t>
@@ -3408,7 +3451,6 @@
           <t>4.9</t>
         </is>
       </c>
-      <c r="F17" t="inlineStr"/>
       <c r="G17" t="inlineStr">
         <is>
           <t>design@divya-consultants.com</t>
@@ -3456,14 +3498,11 @@
           <t>5</t>
         </is>
       </c>
-      <c r="F18" t="inlineStr"/>
-      <c r="G18" t="inlineStr"/>
       <c r="H18" t="inlineStr">
         <is>
           <t>Kishor Choudhari|https://in.linkedin.com/in/kishor-choudhari-a3a59063</t>
         </is>
       </c>
-      <c r="I18" t="inlineStr"/>
       <c r="J18" t="inlineStr">
         <is>
           <t>https://in.linkedin.com/in/kishor-choudhari-a3a59063</t>
@@ -3508,7 +3547,6 @@
 Nagpur"</t>
         </is>
       </c>
-      <c r="G19" t="inlineStr"/>
       <c r="H19" t="inlineStr">
         <is>
           <t>Junaid Ahmed|https://in.linkedin.com/in/junaid-ahmed-0283082b4</t>
@@ -3546,14 +3584,11 @@
           <t>4.5</t>
         </is>
       </c>
-      <c r="F20" t="inlineStr"/>
-      <c r="G20" t="inlineStr"/>
       <c r="H20" t="inlineStr">
         <is>
           <t>Arpit Veldi|https://in.linkedin.com/in/arpit-veldi-573a15a8</t>
         </is>
       </c>
-      <c r="I20" t="inlineStr"/>
       <c r="J20" t="inlineStr">
         <is>
           <t>https://in.linkedin.com/in/sangharshal</t>
@@ -3586,8 +3621,6 @@
           <t>4.6</t>
         </is>
       </c>
-      <c r="F21" t="inlineStr"/>
-      <c r="G21" t="inlineStr"/>
       <c r="H21" t="inlineStr">
         <is>
           <t>Steve Mann|https://www.linkedin.com/in/steve-mann-71971041</t>
@@ -3598,7 +3631,919 @@
           <t>https://ie.linkedin.com/company/mann-engineering</t>
         </is>
       </c>
-      <c r="J21" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J21"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Company</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Website</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Phone</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Address</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Rating</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Email</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>CEO</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Company LinkedIn</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>Leadership LinkedIn</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Abhi Engineering Corporation Pvt Ltd</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>http://abhiengineering.com//</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>+91 712 663 2808</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>404,405, law college square, W High Ct Rd, Master Colony, Tilak Nagar, Gokulpeth, Nagpur, Maharashtra 440010, India</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>4.5</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>bhim Nidwancha|https://in.linkedin.com/in/bhim-nidwancha-2bb79236</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>https://in.linkedin.com/in/rajesh-vishwkarma-00ba67152</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Paramount Engineering Company MIDC Nagpur</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>http://www.paramountengg.com/</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>+91 7104 329 262</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>42W4+53J, Wadi, Nagpur, Maharashtra 440016, India</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>4.7</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Not Acceptable!</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>ROHIT TAPADIA|https://in.linkedin.com/in/rohit-tapadia-ba875a27</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>https://my.linkedin.com/company/paramount-engineering</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>https://in.linkedin.com/in/chetan-sontakke-65152665</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Central India Engineering Pvt Ltd</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>+91 73501 33335</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>F39 Tatya Tope Nagar, WHC Road, near Sai Catering Bichhayat Decorations, Maharashtra 440015, India</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>4.7</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Jatin D. Rathi|https://in.linkedin.com/in/jatin-d-rathi-4a06a062</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>https://in.linkedin.com/in/jatin-d-rathi-4a06a062</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Atlantis Engineers</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>http://atlantisengineers.com/</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>+91 98236 25317</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Little Flowers Nursery School, 172, Mohan Nagar, Nagpur, Maharashtra 440001, India</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>4.3</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Not Acceptable!</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>George Efremidis|https://gr.linkedin.com/in/george-efremidis-3a80a05</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/atlantisengineering/</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Techture</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>http://www.techture.global/</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>+91 91300 92843</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>30, behind Kotak Mahindra Bank, Shankar Nagar, East Shankar Nagar, Nagpur, Maharashtra 440010, India</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>4.1</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Techture offers advanced VDC &amp; BIM services for design, planning, and construction efficiency. Drive accuracy and collaboration. Connect with us today!</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>contact@techture.global</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Muhammad Zubair Khan|https://www.linkedin.com/in/zubairkh</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/techturestructures</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/arnavjain92</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>SD ENGINEERING</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>http://sdstonesengineering.com/</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>+91 84593 16306</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Flat No 104 Tulip Apartment Ram Krishna Nagari New Narsara Road Opp Indian, Gas Godown, Nagpur, Maharashtra 440034, India</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>4.8</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>SD Engineering</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Baasansuren Boris|https://mn.linkedin.com/in/baasansuren-boris-4561a214</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/sdengineering</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Shree Om Sai Construction Nitishka Pvt Ltd - Building Construction</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>https://soscnpltd.in/</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>+91 91752 66870</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>plot no 402, opposite Jaswant tuli mall, Near Indora Chowk, Model Town, Nagpur, Maharashtra 440014, India</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>4.7</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>soscnpltd</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>info@soscnpltd.in</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Amitesh Arun|https://in.linkedin.com/in/amitesh-arun-007386121</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>BHORE ENGINEERING CONSULTANTS PVT. LTD.</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>https://bhoreengineering.com/</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>+91 93212 35472</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>38, Khamla Rd, Near Tajshree Honda, Ramakrishna Nagar, Vivekanand Nagar, Nagpur, Maharashtra 440015, India</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>4.7</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Bhore Engineering Consultants – BEC</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>cvbhore@gmail.com</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Dr. Chaitanya V. Bhore|https://in.linkedin.com/in/chaitanyavbhore</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>https://in.linkedin.com/company/bhore-engineering-consultants-pvt-ltd</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>https://in.linkedin.com/in/chaitanyavbhore</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>OneClick BIM Private Limited</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>http://www.oneclickbim.global/</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>+91 87889 46040</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Basant Apartment, 201, Kadbi Square, Clark Town, Nagpur, Maharashtra 440014, India</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>4.8</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Oneclick BIM is Engineering Consultants offers BIM Services, including architectural, structural, civil, CAD, BIM, detailing, and, electrical.</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>abhijeet@oneclickbim.global</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>ABHIJEET P|https://in.linkedin.com/in/abhijeet-ocb</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>https://in.linkedin.com/company/one-click-bim-cad-services-company-india-dubai</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Dhansa Architect and Engineering Consultant</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>+91 80552 19446</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>1ST FLOOR, CHATRAPATI SQUARE, PLOT NO 50, RING ROAD, Gawande layout, Khamla, Nagpur, Maharashtra 440015, India</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>4.9</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Dhansa Architect|https://in.linkedin.com/in/dhansa-architect-047042237</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>https://in.linkedin.com/in/aditya-bhakte-a3b373153</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Rosmith Engineering</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>+91 94049 02636</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>185, Vedant, Dixit Nagar, Nagpur, Maharashtra 440026, India</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>4.8</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Richard Smith Jr|https://www.linkedin.com/in/richard-smith-jr-041a611a3</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/rasmith</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>imaGIS Engineering Solutions Pvt. Ltd</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>http://www.imagis.co.in/</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>+91 712 222 2137</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Plot No. 13, 2, IT Park Rd, near Gayatri Nagar, Subhash Nagar, Pratap Nagar, Nagpur, Maharashtra 440022, India</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>4.6</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Sandeep Shirkhedkar|https://in.linkedin.com/in/sandeep-shirkhedkar-b0271040</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>https://in.linkedin.com/company/imagis-engineering-solutions</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>https://in.linkedin.com/in/imagis-engineering-solutions-private-limited-nagpur-a9273a358</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Sanghi Consulting Engineers India Pvt. Ltd</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>http://sanghigroup.org/</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>+91 712 224 9225</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>101, Laxmi Keshav Apartments, near Park corner, Dhantoli, Nagpur, Maharashtra 440012, India</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>3.9</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>user@domain.com</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>Rohit Francis|https://in.linkedin.com/in/rohit-francis-b12385183</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>https://in.linkedin.com/company/sanghi-consulting-engineers-india-pvt-ltd-</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>https://in.linkedin.com/in/rohit-francis-b12385183</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>PEB BlueLadder EPC Solutions Pvt Ltd | Pre Engineered Building Solutions | PEB Structure Manufacturer In Nagpur</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>http://www.blueladderepc.com/</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>+91 77988 11367</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>6th Floor, Landmark building, Ramdaspeth, Nagpur, Maharashtra 440010, India</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>4.1</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Leading PEB manufacturer and EPC solution provider in India. Industrial sheds, warehouses, and turnkey construction services.</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Sagar Kewalramani|https://in.linkedin.com/in/sagar-kewalramani-1a0979155</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>https://in.linkedin.com/company/blueladder-epc-solutions</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>https://in.linkedin.com/in/sagar-kewalramani-1a0979155</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Patankar Consultants Pvt. Ltd</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>http://www.patankarconsultants.com/</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>+91 712 224 9293</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>79, Universal Annex,, Shivaji Nagar, Nagpur, Maharashtra 440010, India</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>4.6</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>project@patankarconsultants.com</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>P S Patankar|https://in.linkedin.com/in/p-s-patankar-1576a764</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>https://in.linkedin.com/company/patankar-consultants-pvt-ltd</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>https://in.linkedin.com/in/p-s-patankar-1576a764</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Divya Consultants</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>http://divyaconsultants.in/</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>+91 712 276 6143</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>303, Aarna Complex, Darodkar Square, Central Ave, Ladpura, Itwari, Nagpur, Maharashtra 440002, India</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>4.9</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>design@divya-consultants.com</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>Divya Gupta|https://www.linkedin.com/in/gridsconsulting</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>https://in.linkedin.com/company/divya-consultants</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>https://in.linkedin.com/in/divya-chavan-bb2142118</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Vishwa MEP Engineers Pvt.Ltd</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>https://vishwa.co/</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>+91 712 660 6535</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>43W4+R6P, Ravinagar Square, Yashwant Nagar, Nagpur, Maharashtra 440033, India</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>Kishor Choudhari|https://in.linkedin.com/in/kishor-choudhari-a3a59063</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>https://in.linkedin.com/in/kishor-choudhari-a3a59063</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Ahmad Construction &amp; Interiors</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/ahmad_construction_interiors?igsh=enR0YTFmampnczRw</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>+91 76209 28833</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>102, Aman's Villa, Eidgh Ground, above Shahu Kirana, Adarsh Colony, Jafar Nagar, New Mankapur, Nagpur, Maharashtra 440013, India</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>4.9</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>384 Followers, 1,096 Following, 40 Posts - Osman Furniture &amp; Interior (@ahmad_construction_interiors) on Instagram: "Contact Us:-7620928833
+Building Construction,⚒️
+Interior Design
+Modular Furniture
+Civil Engg Drawing🏙️
+Architectural Planning💻 
+3d View
+Nagpur"</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>Junaid Ahmed|https://in.linkedin.com/in/junaid-ahmed-0283082b4</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>https://pk.linkedin.com/company/accopakistan</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>https://in.linkedin.com/in/afzaal-ahmad-136044307</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>DUSON CIVIL ENGINEERING SERVICES LLP</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>+91 712 224 3354</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>35, Khamla Rd, Deo Nagar, Nagpur, Maharashtra 440015, India</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>4.5</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>Arpit Veldi|https://in.linkedin.com/in/arpit-veldi-573a15a8</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>https://in.linkedin.com/in/sangharshal</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Mann Engineering Company</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>http://mannengineeringcompany.com/</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>+91 99227 00037</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Kamptee Rd, Pili Nadi, Nagpur, Maharashtra 440026, India</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>4.6</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>Steve Mann|https://www.linkedin.com/in/steve-mann-71971041</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>https://ie.linkedin.com/company/mann-engineering</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Improved the industry searching algorithm
</commit_message>
<xml_diff>
--- a/company_leads.xlsx
+++ b/company_leads.xlsx
@@ -17,6 +17,7 @@
     <sheet name="CodePilot AI1" sheetId="8" state="visible" r:id="rId8"/>
     <sheet name="CodePilot AI2" sheetId="9" state="visible" r:id="rId9"/>
     <sheet name="gg" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Healthcare AI" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1481,6 +1482,984 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J21"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Company</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Website</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Phone</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Address</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Rating</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Email</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>CEO</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Company LinkedIn</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>Leadership LinkedIn</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>ArrayGen Technologies Pvt Ltd</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>https://www.arraygen.com/</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>+91 96736 25446</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Office No 237,Second Floor, VTP Trade Park, URBAN NEST, Wing 4, Shree Siddhivinayak Meera, Undri, Pune, Maharashtra 411060, India</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>4.7</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Bioinformatics data analysis, next generation sequencing, Sequencing Services, Microarray data analysis, Agilent, NGS, data analysis course, genomics service provider, Bioinformatics courses, Data Analysis, Annotation, custom microarray, Biotech company,</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr"/>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Rajesh Mahato|https://in.linkedin.com/in/rajesh-mahato-06158518</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>https://in.linkedin.com/company/arraygen-technologies</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>IshVed</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>https://ishved.com/</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>+91 83296 95476</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Gera's Imperium Alpha, Rajaram Patil Nagar, Vitthal Nagar, Kharadi, Pune, Maharashtra 411014, India</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>4.7</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr"/>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>info@ishved.com</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Dr. Sanjay Wayal|https://in.linkedin.com/in/dr-sanjay-wayal-857b8225</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>https://in.linkedin.com/company/ishved</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>https://in.linkedin.com/in/ishved-group-a28156211</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>geneOmbio Technologies Pvt Ltd.</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>http://www.geneombiotechnologies.com/</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>+91 99600 00984</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Office No 302, Lalani Quantum, Patil Nagar, Bavdhan, Pune, Maharashtra 411021, India</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>4.6</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>geneOmbio</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>crs@geneombiotechnologies.com</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Bikash Aich|https://in.linkedin.com/in/bikash-aich-3840ab8</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>https://in.linkedin.com/company/geneombio-technologies</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>ADEETECHGENE BIOTECH PVT LTD</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>http://www.adeetech.com/</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>+91 99214 46321</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>A8 Thorve, Vishva commercial, Balewadi, Pune, Maharashtra 411069, India</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>4.9</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADEETECH is Biotech B2B Company with current services on COVID19 Clinical Trials, USFDA Rapid kits, BSL2 and BSL3 Lab setup, Coronavirus antiviral research  </t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>adeetechgene@gmail.com</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Devendra Lingojwar|https://in.linkedin.com/in/devendra-lingojwar-71378039</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>https://in.linkedin.com/company/adeetech</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>https://in.linkedin.com/in/devendra-lingojwar-71378039</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Astranova Biotech Pvt Ltd | Pharmaceutical Company in Pune</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>+91 84594 61724</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>B-104, 1st Floor, City Vista, Kolte Patil Downtown, Fountain Road, Ashoka Nagar, Kharadi, Pune, Maharashtra 411014, India</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>4.8</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr"/>
+      <c r="G6" t="inlineStr"/>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Santosh Sangale|https://in.linkedin.com/in/santosh-sangale-b9a63a191</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>https://in.linkedin.com/company/astranova-biotech-pvt-ltd</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>https://in.linkedin.com/in/santosh-sangale-b9a63a191</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Nirav Biosolutions Pvt. Ltd. - A Biotechnology Resource Center</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>https://www.niravbiosolutions.com/</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr"/>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Unit no. FRZ 02, Reliance Mall, BRS No. 169/1, DP Rd, next to WESTEND MALL, Ward No. 8, Sector II, Aundh, Pune, Maharashtra 411067, India</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>4.7</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Explore the story and mission behind Nirav Biosolutions, a leading supplier-distributor in the field of biotechnology. Discover our team of experts, cutting-edge projects, and commitment to biotechnology. Learn how Nirav Bio Solutions is making a positive impact on biotechnology.</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>inquiry@niravbiosolutions.net</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Pravin Sharma|https://in.linkedin.com/in/pravin-sharma-27191221</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>https://in.linkedin.com/company/nirav-biosolutions-pvt-ltd</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>https://in.linkedin.com/in/nirav-biosolutions-14054545</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Hi Tech Biosciences India Private Limited</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>http://www.htblindia.com/</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>+91 20 2528 5426</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>S No, Saudamini complex, C-2, Unit 102+103, 101/1, Paud Rd, Kothrud, Pune, Maharashtra 411038, India</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>4.2</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Hi Tech Biosciences India Ltd.</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>info@htblindia.com</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Vinay_Bhaiya Dhanale|https://in.linkedin.com/in/vinay-bhaiya-dhanale-7370b920</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>https://in.linkedin.com/company/hi-tech-biosciences-india-private-limited</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>https://in.linkedin.com/in/hi-tech-biosciences-india-private-limited-679996307</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Kan Biosys Pvt Ltd</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>http://www.kanbiosys.com/</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>+91 20 2439 1779</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>917/17, Raveedeep, Prin, K R, Professor Keshav Ramchandra Kanitkar Path, off Fergusson College Road, Ganeshwadi, Deccan Gymkhana, Pune, Maharashtra 411004, India</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>4.3</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Home - Kan Biosys</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>connect@kanbiosys.com</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Sandeepa Kanitkar|https://in.linkedin.com/in/sandeepakanitkar-kanbiosys</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>https://in.linkedin.com/company/kanbiosys-pvt-ltd</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>BioResource Biotech Pvt. Ltd.</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>http://bioresourcebiotech.com/</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>+91 20 2589 6379</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Plot # 18/1, Madhukunj Society, Off, Pashan Rd, Panchawati, Pune, Maharashtra 411008, India</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>4.2</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr"/>
+      <c r="G10" t="inlineStr"/>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Jagannath Sonavane|https://in.linkedin.com/in/jagannath-sonavane-b7349714</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>https://in.linkedin.com/company/bioresouce-biotech-pvt.ltd.</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>https://in.linkedin.com/in/jagannath-sonavane-b7349714</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Enzene Biosciences Limited</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>http://www.enzene.com/</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>+91 20 6718 4200</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Plo Number Number 165, Priyadarshani Society 26, 1/26, Internal Rd, next to Gujjar Bharath gas) T, MIDC, Bhosari, Pune, Pimpri-Chinchwad, Maharashtra 411026, India</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>4.4</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr"/>
+      <c r="G11" t="inlineStr"/>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Not Available</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/enzene</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/kumar-bala-5225326</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Ajay Biotech (India) Ltd.</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>https://ajaybiotech.com/</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>+91 98237 31990</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>No 107 Plot No, Netsurf, 3rd floor, Sr, 2, Baner Rd, Baner, Pune, Maharashtra 411045, India</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>4.9</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>We are the leading manufacturer of Agriculture, Public Health, Personal Hygiene, Veterinary, Fishery and Medical Device.</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>enquiry@ajaybio.in</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Dr Subrata Sarkar|https://in.linkedin.com/in/dr-subrata-sarkar-30ba9649</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>https://in.linkedin.com/company/ajay-biotech-india-ltd</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>https://in.linkedin.com/in/ajay-ajay-443499305</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>GeneSpectrum Life Sciences LLP</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>https://genespectrum.in/</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>+91 70213 86045</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Sunit Riddhi Siddhi Building, 104, Sinhgad Rd, off PL Deshpande Garden, Sarita Vihar Phase 2, Dattawadi, Pune, Maharashtra 411030, India</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>4.7</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>GeneSpectrum - Simplifying Bioinformatics - GeneSpectrum Life Sciences</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>contact@genespectrum.in</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Dr. Bhavin Patel|https://in.linkedin.com/in/dr-bhavin-patel-09a13a22</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>https://in.linkedin.com/company/genespectrum</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Thopte Biotech Pvt. Ltd</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>http://www.thoptebiotech.com/</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>+91 98348 35706</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>No. 198, Shriram Sahakari Society, Sahakar Nagar, No. 1, near Kamgar Kalyan Mandal, Pune, Maharashtra 411009, India</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Not Acceptable!</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr"/>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>Sampat Thopte|https://in.linkedin.com/in/sampat-thopte-34104a49</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>https://in.linkedin.com/company/thopte-biotech-private-limited</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>https://in.linkedin.com/in/sampat-thopte-34104a49</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>GREEN PYRAMID BIOTECH PVT. LTD</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>http://www.greenpyramidbiotech.com/</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr"/>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Incubation Center, NCL Innovation park, Dr Homi Bhabha Rd, Pashan, Pune, Maharashtra 411008, India</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>4.3</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Experience Green Pyramid Biotech, a sustainable leader in wellness solutions. Explore our eco-friendly products for a healthier lifestyle.</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>info@greenpyramidbiotech.com</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Asmita Prabhune|https://in.linkedin.com/in/asmita-prabhune-01580732</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>https://in.linkedin.com/company/green-pyramid-biotech-pvt-ltd</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>https://in.linkedin.com/in/asmita-prabhune-1601037</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>TCG International Biotech Park</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>+91 20 6790 3900</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Genesis Square, Ground Floor Rajiv Gandhi Infotech - Biotech Park, MIDC, Hinjawadi Phase II, Hinjawadi, Pune, Maharashtra 411057, India</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>4.5</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr"/>
+      <c r="G16" t="inlineStr"/>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>Prasanta K Biswal|https://in.linkedin.com/in/prasantakbiswal</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>https://in.linkedin.com/company/tcg-international-biotech-park-ltd</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Amalgam Biotech: Bio Culture for Wastewater (ETP &amp; STP) &amp; Odour Control Experts [Manufacturer &amp; Service Provider]</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>https://www.amalgambiotech.com/</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>+91 72760 20758</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Amalgam Biotech, Prayag, Lane Number 7, next to Saipro Building, behind Moze College, Laxman Nagar, Baner, Pune, Maharashtra 411045, India</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>4.8</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Amalgam Biotech offers advanced bioculture for wastewater treatment – ideal for STPs, ETPs, bio-toilets &amp; industrial use. Trusted by top brands.</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>sales@amalgambiotech.com</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>Not Available</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>https://in.linkedin.com/company/amalgam-biotech</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>SEZ Biotech Services</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>+91 97189 71895</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>GX87+83, Taluka Haveli, SERUM INSTITUTE OF INDIA-1, Amanora Park Town Main Rd, Manjari Budruk, Pune, Maharashtra 412307, India</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>4.6</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr"/>
+      <c r="G18" t="inlineStr"/>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>Bathina seshagiri|https://in.linkedin.com/in/bathina-seshagiri-4b33209</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/biotech-service</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>BioSphere LifeSciences Pvt. Ltd</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>+91 20 6529 0294</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>1st Floor, Plot # 18/1, Madhukunj Society,, Pashan Rd, Panchawati, Pune, Maharashtra 411008, India</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>4.3</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr"/>
+      <c r="G19" t="inlineStr"/>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>Dinesh Dhage|https://in.linkedin.com/in/dinesh-dhage-0b135a153</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>https://in.linkedin.com/company/biosphere-lifesciences-pvt-ltd</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>https://in.linkedin.com/in/rajnikant-date-801ab1121</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Aamikza Biotechnology Pvt. Ltd. (Research and Innovation Centre)</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>https://aamikza.com/</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr"/>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>ESD House, Plot No. 55, Hadapsar Industrial Estate, Hadapsar, Pune, Maharashtra 411013, India</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>We’re pioneering the cultivation of strains to craft fermented milk products with precise applications. Did you know, references to dairy and milk products can be traced back to the Rigveda, an ancient Indian scripture believed to have been written around 1700 BCE? At our core, we honor India’s rich traditions – even our name, Aamikza, is derived from ‘Aamixa,’ a Sanskrit term for fermentation.</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>info@aamikza.com</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>Amruta Pawar|https://in.linkedin.com/in/amruta-pawar-545797233</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/aamikza-biotechnology-pvt-ltd</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>https://in.linkedin.com/in/dr-dolly-patel-610bb4312</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>MrBiologist Pune</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>https://www.askmrbiologist.com/</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr"/>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>2nd floor, Shivam enterprise, S no 36 /1/1, Sinhgad Rd, near greenfield hotel, Vadgaon Khurd, Nanded Fata, Pandurang Industrial Area, Nanded, fats, Pune, Maharashtra 411068, India</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>4.9</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Experience advancement with Mr Biologist - North East India's premier Contract Research Organisation specializing in computational biology, molecular biology, and bioinformatics services.</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr"/>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>Amrit Pritam Bhuyan|https://in.linkedin.com/in/amrit-pritam-bhuyan-31a63b69</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>https://in.linkedin.com/company/mrbiologist</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>https://in.linkedin.com/in/amrit-pritam-bhuyan-31a63b69</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
fixed the chat section issue
</commit_message>
<xml_diff>
--- a/company_leads.xlsx
+++ b/company_leads.xlsx
@@ -17,6 +17,8 @@
     <sheet name="CodePilot AI1" sheetId="8" state="visible" r:id="rId8"/>
     <sheet name="CodePilot AI2" sheetId="9" state="visible" r:id="rId9"/>
     <sheet name="gg" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Chatbot AI2" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="Chatbot AI3" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1481,6 +1483,138 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Company</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Website</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Phone</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Address</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Rating</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Email</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>CEO</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Company LinkedIn</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>Leadership LinkedIn</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Company</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Website</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Phone</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Address</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Rating</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Email</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>CEO</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Company LinkedIn</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>Leadership LinkedIn</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
side bar complete fix
</commit_message>
<xml_diff>
--- a/company_leads.xlsx
+++ b/company_leads.xlsx
@@ -17,6 +17,7 @@
     <sheet name="CodePilot AI1" sheetId="8" state="visible" r:id="rId8"/>
     <sheet name="CodePilot AI2" sheetId="9" state="visible" r:id="rId9"/>
     <sheet name="gg" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="AutoFlow AI" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1481,6 +1482,72 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Company</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Website</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Phone</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Address</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Rating</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Email</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>CEO</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Company LinkedIn</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>Leadership LinkedIn</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>